<commit_message>
Update Rocket21 affiliate pool (2026-08-04 23:20)
</commit_message>
<xml_diff>
--- a/affiliate_data/rocket_curated.xlsx
+++ b/affiliate_data/rocket_curated.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Curated Products" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Curated Products'!$A$1:$L$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Curated Products'!$A$1:$L$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -515,7 +515,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>ของเล่นโมเดลรถถังทหาร เครื่องบินทหาร สำหรับเด็ก ของเล่นบล็อคตัวต่อฝึกเสริมสมาธิ</t>
+          <t>MEIYIJIA เครื่องดูดฝุ่นในรถ ไร้สาย 12000Pa car vacuum cleaner เครื่องดูดฝุ่นขนาดเล็ก ที่ดูดฝุ่นในรถยนต์ ภายในบ้าน เตียง</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
@@ -527,7 +527,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/20uOne6kLC</t>
+          <t>https://s.shopee.co.th/7Kvv9iFNqe</t>
         </is>
       </c>
       <c r="K2" s="2" t="n"/>
@@ -539,7 +539,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>สินค้าใหม่ 2026 scale 1:72 โมเดลประกอบ บล็อก ตัวต่อ รถทหาร รถถัง T90 T14 M1A2 เครื่องบิน</t>
+          <t>แบตเตอรี่ 12V 8AH/12AH UPS ไฟฉุกเฉิน เครื่องมือเกษตร ใส่เครื่องพ่นยา สินค้าพร้อมส่งในไทย</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr"/>
@@ -551,7 +551,7 @@
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/AAG6Wfo2Uy</t>
+          <t>https://s.shopee.co.th/9pdG8KMRW0</t>
         </is>
       </c>
       <c r="K3" s="2" t="n"/>
@@ -563,7 +563,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>โมเดลรถถังอาวุธทหาร UK US WW2 ของเล่นสําหรับเด็ก ของขวัญวันเกิด 524 ชิ้น Sluban 0858</t>
+          <t>แบตเตอรี่12V 20Ah แบตเตอรี่แห้งแท้ รุ่น 6-DZF-20 แบตรถสามล้อไฟฟ้า รถจักรยานไฟฟ้า จักรยานไฟฟ้า,สกู๊ตเตอร์ สามล้อไฟฟ้า</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
@@ -575,7 +575,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2VqfObCYkg</t>
+          <t>https://s.shopee.co.th/8fRIkCQTpy</t>
         </is>
       </c>
       <c r="K4" s="2" t="n"/>
@@ -587,7 +587,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>ProudNada Toys ตัวต่อ ทหาร รถถัง รถหุ้มเกราะ SLUBAN MODEL BRICKS M4A3(76W) MEDIUM TANK 715 PCS M38-B1110</t>
+          <t>แบตเตอรี่ลิเธียม 12V 10AH/22AH แบตเตอรี่ สามารถชาร์จโดยใช้พลังงานแสงอาทิตย์แล แบตเตอรี่เครื่องพ่นสารเคมี แบตเตอรี</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr"/>
@@ -599,7 +599,7 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5q77Mkho5s</t>
+          <t>https://s.shopee.co.th/70J4l9fhZH</t>
         </is>
       </c>
       <c r="K5" s="2" t="n"/>
@@ -611,7 +611,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>M2 Bradley รถหุ้มเกราะทหารราบ เข้ากันได้ตัวต่อเลโก้ 1862ชิ้น 12GO Tank โมเดลประกอบแล้ว</t>
+          <t>แบตเตอรี่12V 20Ah แบตเตอรี่แห้งแท้ รุ่น 6-DZF-20 แบตรถสามล้อไฟฟ้า รถจักรยานไฟฟ้า จักรยานไฟฟ้า,สกู๊ตเตอร์ สามล้อไฟฟ้า</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
@@ -623,7 +623,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1Vy8CoShJr</t>
+          <t>https://s.shopee.co.th/8pkiwXqoKq</t>
         </is>
       </c>
       <c r="K6" s="2" t="n"/>
@@ -635,7 +635,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>CH-53E เฮลิคอปเตอร์ทหาร เข้ากันได้ตัวต่อเลโก้ 2192ชิ้น Reobrix Plane โมเดลประกอบแล้ว</t>
+          <t>เครื่องดูดฝุ่นในรถยนต์ เครื่องดูดฝุ่นไร้สาย แรงดูดสูง 99000Pa เครื่องดูดฝุ่นพกพา ชาร์จUSB ส่งด่วนจากไทย</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr"/>
@@ -647,7 +647,7 @@
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2BDp03Gt5Y</t>
+          <t>https://s.shopee.co.th/7Kvv9o8M0p</t>
         </is>
       </c>
       <c r="K7" s="2" t="n"/>
@@ -659,7 +659,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>สินค้าใหม่ปี 2026 โมเดลเครื่องบิน เฮลิคอปเตอร์ f35 f16 j10 f14 รถทหาร ทหาร</t>
+          <t>เครื่องดูดฝุ่นมือถือ350วัตต์ไร้สายที่มีประสิทธิภาพพายุไซโคลนดูดแบบพกพาชาร์จเครื่องดูดฝุ่น ไร้สาย ที่ดูดฝุ่น ดูดฝุ่นในรถ</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
@@ -671,7 +671,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9fJpvqwjNy</t>
+          <t>https://s.shopee.co.th/5LAqm9OQqo</t>
         </is>
       </c>
       <c r="K8" s="2" t="n"/>
@@ -683,7 +683,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>ProudNada Toys ของเล่นเด็ก ตัวต่อ เฮลิคอปเตอร์ ทหาร Sluban Model Bricks KA-50 330 PCS B0752</t>
+          <t>ที่ใส่ก้านกันสาด ฐานเสาดัก Tarp Pole Fixator มีน็อตคู่ แบบปรับได้ หลากสีอุปกรณ์เสริม สําหรับตั้งเต็นท์</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr"/>
@@ -695,7 +695,7 @@
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/qiRPdUIZW</t>
+          <t>https://s.shopee.co.th/8pkiwbFNXY</t>
         </is>
       </c>
       <c r="K9" s="2" t="n"/>
@@ -707,7 +707,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>โมเดลกระดาษประกอบเครื่องบินขนส่งทหาร AC-130U Spooky Gunship - MohinhgiayVN</t>
+          <t>ตัวล็อคฮุคแขวนสินค้า ระบบแม่เหล็ก สีแดง ขนาด 4 5 6 7 8 mm สำหรับร้านค้า ร้านไอที</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
@@ -719,7 +719,7 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5VUGyE2MpD</t>
+          <t>https://s.shopee.co.th/2VqfOyh4Z1</t>
         </is>
       </c>
       <c r="K10" s="2" t="n"/>
@@ -731,7 +731,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>MOC Assembly Toy Army ZU-23-2 โมเดลทหาร</t>
+          <t>BONMECOM2 / ปลั๊กไฟ Melon/ ปลั๊กไฟโต๊ะคอม/ ปลั๊กไฟโต๊ะทำงาน 2 ช่อง 1 สวิตซ์ 3USB (1.5M) มี มอก. (ของแถมคละสี)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr"/>
@@ -743,7 +743,7 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9fJpvts59O</t>
+          <t>https://s.shopee.co.th/3qM2zRT4Ho</t>
         </is>
       </c>
       <c r="K11" s="2" t="n"/>
@@ -755,7 +755,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>MOC Assembly Toy Army LAV-25 โมเดลทหาร</t>
+          <t>ปลั๊กไฟ 3 4 5 ช่อง 2300 W ปลั๊กพ่วง สายยาว 3 เมตร 5 เมตร8 เมตร</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
@@ -767,7 +767,7 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2BDp08NfRA</t>
+          <t>https://s.shopee.co.th/2VqfP0SeYX</t>
         </is>
       </c>
       <c r="K12" s="2" t="n"/>
@@ -779,7 +779,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>MOC Assembly Toy Army ZSU-234 โมเดลทหาร</t>
+          <t>ปรับปรุงใหม่และเพิ่มความหนาขึ้นปลั๊กสนาม 2x4 บล็อกยาง สาย VCT2x1 รองรับไฟสูงสุด 3000W ยาว 5M,10M,15M,20M,30M</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
@@ -791,7 +791,7 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6L3Nxnyo90</t>
+          <t>https://s.shopee.co.th/5LAqmFdXSe</t>
         </is>
       </c>
       <c r="K13" s="2" t="n"/>
@@ -803,7 +803,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>บล็อกตัวต่อโมเดลฟิกเกอร์ รูปเมืองทหาร ยาว 1x16 Diy ของเล่นสร้างสรรค์ ของขวัญ 5 ชิ้น</t>
+          <t>ปลั๊กไฟ 3/5 รู, หลายเต้ารับ, แถบสายไฟต่อ, ปลั๊กสายไฟต่อ, แจ็คชาร์จไฟ USB, รางปลั๊กไฟ, สายยาว 2/3/5M เมตร</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
@@ -815,7 +815,7 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1qaybYARpE</t>
+          <t>https://s.shopee.co.th/4fv9z2cEeM</t>
         </is>
       </c>
       <c r="K14" s="2" t="n"/>
@@ -827,7 +827,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>4D MODEL โมเดลหุ่นทหารมินิ หุ่นจำลอง สินค้าแท้ ลิขสิทธิ์ถูกต้อง Miniature assembly special Troops Army Figures MMXJ-98</t>
+          <t>ปลั๊กพ่วง ปลั๊กสนาม 2x4 บล็อกยาง สาย VCT 24sq.mm รองรับไฟสูงสุด 3000W ยาว 5M,10M,15M,20M หุ้มยางต่อสายไฟ สายไฟหุ้มฉนวน</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr"/>
@@ -839,7 +839,7 @@
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5ArQZgxlab</t>
+          <t>https://s.shopee.co.th/7VFLMGHDMA</t>
         </is>
       </c>
       <c r="K15" s="2" t="n"/>
@@ -851,7 +851,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>โมเดลฟิกเกอร์ทหารทหารทหาร ขยับข้อต่อได้ ของเล่นสําหรับเด็กผู้ชาย</t>
+          <t>Deli ปลั๊กไฟ ปลั๊กแปลง ปลั๊กสากล ปลั๊กสามตา ไฟ 10A 2500W ทนความร้อนได้ 750องศา Universal Adapter</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
@@ -863,7 +863,7 @@
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/60QXZFDEUS</t>
+          <t>https://s.shopee.co.th/3qM2zXPotA</t>
         </is>
       </c>
       <c r="K16" s="2" t="n"/>
@@ -875,7 +875,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>MEIYIJIA เครื่องดูดฝุ่นในรถ ไร้สาย 12000Pa car vacuum cleaner เครื่องดูดฝุ่นขนาดเล็ก ที่ดูดฝุ่นในรถยนต์ ภายในบ้าน เตียง</t>
+          <t>ปลั๊กไฟพ่วงกลม 5 ช่อง 3 USB ความยาว 3 ,5, 8 เมตร</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr"/>
@@ -887,7 +887,7 @@
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7Kvv9iFNqe</t>
+          <t>https://s.shopee.co.th/7Kvv9z3MQv</t>
         </is>
       </c>
       <c r="K17" s="2" t="n"/>
@@ -899,7 +899,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>แบตเตอรี่ 12V 8AH/12AH UPS ไฟฉุกเฉิน เครื่องมือเกษตร ใส่เครื่องพ่นยา สินค้าพร้อมส่งในไทย</t>
+          <t>เก้าอี้แคมป์ปิ้ง พนักพิงสูง เก้าอี้สนาม พับได้ แบบพกพา ปิคนิค แถมถุงเก็บ รับน้ำหนัก 300KG</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
@@ -911,7 +911,7 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9pdG8KMRW0</t>
+          <t>https://s.shopee.co.th/AAG6XCsmzJ</t>
         </is>
       </c>
       <c r="K18" s="2" t="n"/>
@@ -923,7 +923,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>แบตเตอรี่12V 20Ah แบตเตอรี่แห้งแท้ รุ่น 6-DZF-20 แบตรถสามล้อไฟฟ้า รถจักรยานไฟฟ้า จักรยานไฟฟ้า,สกู๊ตเตอร์ สามล้อไฟฟ้า</t>
+          <t>WTHB เก้าอี้แคมป์ปิ้ง เพิ่มผ้าฝ้าย พนักพิงสูง เก้าอี้สนาม เก้าอี้สนามพับได้ ปิคนิค รับน้ำหนัก 300KG</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr"/>
@@ -935,7 +935,7 @@
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8fRIkCQTpy</t>
+          <t>https://s.shopee.co.th/4fv9z7LZZT</t>
         </is>
       </c>
       <c r="K19" s="2" t="n"/>
@@ -947,7 +947,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>แบตเตอรี่ลิเธียม 12V 10AH/22AH แบตเตอรี่ สามารถชาร์จโดยใช้พลังงานแสงอาทิตย์แล แบตเตอรี่เครื่องพ่นสารเคมี แบตเตอรี</t>
+          <t>ซื้อ 1 แถม1ไฟฉายคาดหัว ไฟคาดหัว ส่องไกล ไฟคาดหัว LED ส่องกบ เดินป่า ลุยฝนได้ สว่างมาก รับประกันความสว่า</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
@@ -959,7 +959,7 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/70J4l9fhZH</t>
+          <t>https://s.shopee.co.th/1Vy8DJSgdv</t>
         </is>
       </c>
       <c r="K20" s="2" t="n"/>
@@ -971,7 +971,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>แบตเตอรี่12V 20Ah แบตเตอรี่แห้งแท้ รุ่น 6-DZF-20 แบตรถสามล้อไฟฟ้า รถจักรยานไฟฟ้า จักรยานไฟฟ้า,สกู๊ตเตอร์ สามล้อไฟฟ้า</t>
+          <t>20warehouse ไฟฉายคาดศีรษะ LED 90 Lumens ปรับมุมได้ ไฟส่องสว่างพกพา สำหรับเดินป่า กรีดยาง ซ่อมรถ ตกปลา</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr"/>
@@ -983,7 +983,7 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8pkiwXqoKq</t>
+          <t>https://s.shopee.co.th/40fTBvEz6Q</t>
         </is>
       </c>
       <c r="K21" s="2" t="n"/>
@@ -995,7 +995,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>เครื่องดูดฝุ่นในรถยนต์ เครื่องดูดฝุ่นไร้สาย แรงดูดสูง 99000Pa เครื่องดูดฝุ่นพกพา ชาร์จUSB ส่งด่วนจากไทย</t>
+          <t>ซื้อ1แถม1ไฟฉายแรงสูง ไฟฉายLED ไฟฉายพกพา ชาร์จUSB ส่องสว่างไกล ปรับได้5ระดับ</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
@@ -1007,7 +1007,7 @@
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7Kvv9o8M0p</t>
+          <t>https://s.shopee.co.th/9fJpwLobn1</t>
         </is>
       </c>
       <c r="K22" s="2" t="n"/>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>เครื่องดูดฝุ่นมือถือ350วัตต์ไร้สายที่มีประสิทธิภาพพายุไซโคลนดูดแบบพกพาชาร์จเครื่องดูดฝุ่น ไร้สาย ที่ดูดฝุ่น ดูดฝุ่นในรถ</t>
+          <t>530 Portable Flashlights Miniไฟฉายสว่างมาก CREE LED XPE+COB 2in1 600mah usb charge 3mode ซูมได้</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr"/>
@@ -1031,7 +1031,7 @@
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5LAqm9OQqo</t>
+          <t>https://s.shopee.co.th/2qTVno4nfp</t>
         </is>
       </c>
       <c r="K23" s="2" t="n"/>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>ที่ใส่ก้านกันสาด ฐานเสาดัก Tarp Pole Fixator มีน็อตคู่ แบบปรับได้ หลากสีอุปกรณ์เสริม สําหรับตั้งเต็นท์</t>
+          <t>เชือกรอกปรับระดับได้ เชือกเต็นท์ เชือกรอกปรับระดับได้ 4m สําหรับตั้งแคมป์กลางแจ้ง รอกเชือก เชือกยก</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
@@ -1055,7 +1055,7 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/8pkiwbFNXY</t>
+          <t>https://s.shopee.co.th/1qaybz40f6</t>
         </is>
       </c>
       <c r="K24" s="2" t="n"/>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>ตัวล็อคฮุคแขวนสินค้า ระบบแม่เหล็ก สีแดง ขนาด 4 5 6 7 8 mm สำหรับร้านค้า ร้านไอที</t>
+          <t>สมอบกเหล็กหล่อ สมอบกเต็นท์ วงแหวนเรืองแสง 20/30/40 CM เหล็กคาร์บอนสูง</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr"/>
@@ -1079,7 +1079,7 @@
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2VqfOyh4Z1</t>
+          <t>https://s.shopee.co.th/5fnhB2pljE</t>
         </is>
       </c>
       <c r="K25" s="2" t="n"/>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>BONMECOM2 / ปลั๊กไฟ Melon/ ปลั๊กไฟโต๊ะคอม/ ปลั๊กไฟโต๊ะทำงาน 2 ช่อง 1 สวิตซ์ 3USB (1.5M) มี มอก. (ของแถมคละสี)</t>
+          <t>มีดตั้งแคมป์กลางแจ้ง (สแตนเลส) - มีดอเนกประสงค์แบบพกพา คมชัดเป็นพิเศษ G3204</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr"/>
@@ -1103,7 +1103,7 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3qM2zRT4Ho</t>
+          <t>https://s.shopee.co.th/50Y0Npil9c</t>
         </is>
       </c>
       <c r="K26" s="2" t="n"/>
@@ -1115,7 +1115,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>ปลั๊กไฟ 3 4 5 ช่อง 2300 W ปลั๊กพ่วง สายยาว 3 เมตร 5 เมตร8 เมตร</t>
+          <t>#019 Kershaw #Folding knife #มีดพับ #มีดเดินป่า #มีดเอนกประสงค์ LIFEPLAZA</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr"/>
@@ -1127,7 +1127,7 @@
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2VqfP0SeYX</t>
+          <t>https://s.shopee.co.th/2gA5bYimaj</t>
         </is>
       </c>
       <c r="K27" s="2" t="n"/>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>ปรับปรุงใหม่และเพิ่มความหนาขึ้นปลั๊กสนาม 2x4 บล็อกยาง สาย VCT2x1 รองรับไฟสูงสุด 3000W ยาว 5M,10M,15M,20M,30M</t>
+          <t>NANMEEBOOKS หนังสือ แผนที่ประวัติศาสตร์ เหตุการณ์เปลี่ยนโลก เสริมความรู้</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr"/>
@@ -1151,7 +1151,7 @@
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5LAqmFdXSe</t>
+          <t>https://s.shopee.co.th/6Ajxm0MsFI</t>
         </is>
       </c>
       <c r="K28" s="2" t="n"/>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>ปลั๊กไฟ 3/5 รู, หลายเต้ารับ, แถบสายไฟต่อ, ปลั๊กสายไฟต่อ, แจ็คชาร์จไฟ USB, รางปลั๊กไฟ, สายยาว 2/3/5M เมตร</t>
+          <t>WAYFARER โต๊ะแคมป์กลางแจ้ง โต๊ะพับ โต๊ะไข่เจียว โต๊ะตั้งแคมป์ ซื้อ 1 แถม 1 ถุงจัดส่ง ง่ายต่อการพกพา ทำความสะอาดง่าย</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr"/>
@@ -1175,7 +1175,7 @@
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4fv9z2cEeM</t>
+          <t>https://s.shopee.co.th/5fnhB6BArU</t>
         </is>
       </c>
       <c r="K29" s="2" t="n"/>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>ปลั๊กพ่วง ปลั๊กสนาม 2x4 บล็อกยาง สาย VCT 24sq.mm รองรับไฟสูงสุด 3000W ยาว 5M,10M,15M,20M หุ้มยางต่อสายไฟ สายไฟหุ้มฉนวน</t>
+          <t>MAX FIRE แก๊สกระป๋อง แก๊สปิคนิค พร้อมด้วยระบบป้องกันการระเบิด ปริมาณ 250g. ประเทศเกาหลี 1 แพ็ค</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr"/>
@@ -1199,7 +1199,7 @@
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7VFLMGHDMA</t>
+          <t>https://s.shopee.co.th/6Ajxm1pku2</t>
         </is>
       </c>
       <c r="K30" s="2" t="n"/>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Deli ปลั๊กไฟ ปลั๊กแปลง ปลั๊กสากล ปลั๊กสามตา ไฟ 10A 2500W ทนความร้อนได้ 750องศา Universal Adapter</t>
+          <t>เชือกพาราคอร์ด เชือกตากผ้า เชือก ยาว4/10เมตร เก็บง่าย คุณภาพดี ทนทาน คละสี สำหรับเดินป่า ตั้งแคมป์ ใช้ผูกเอนกประสงค์</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr"/>
@@ -1223,7 +1223,7 @@
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3qM2zXPotA</t>
+          <t>https://s.shopee.co.th/AKZWjhSCbh</t>
         </is>
       </c>
       <c r="K31" s="2" t="n"/>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>ปลั๊กไฟพ่วงกลม 5 ช่อง 3 USB ความยาว 3 ,5, 8 เมตร</t>
+          <t>หมอนเป่าลม หมอนหนุนเป่าลมพกพา เบามาก จัดเก็บง่าย ขนาดพกพา 43x28x12cm หมอนเป่าลม ใบใหญ่ เหมาะสำหรับสำนักงาน การท่องเที่ยว</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr"/>
@@ -1247,7 +1247,7 @@
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/7Kvv9z3MQv</t>
+          <t>https://s.shopee.co.th/4qEaBblIDQ</t>
         </is>
       </c>
       <c r="K32" s="2" t="n"/>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>เก้าอี้แคมป์ปิ้ง พนักพิงสูง เก้าอี้สนาม พับได้ แบบพกพา ปิคนิค แถมถุงเก็บ รับน้ำหนัก 300KG</t>
+          <t>ผ้าบัฟ ผ้าโพกหน้า ทั้งวิ่ง ล่าสัตว์ ตกปลา เดินป่า รถจักรยานยนต์ ปั่นจักรยาน เล่นสกี ชิคสุดๆค่าได้ยาวนานคุ้มค่า</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr"/>
@@ -1271,374 +1271,14 @@
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/AAG6XCsmzJ</t>
+          <t>https://s.shopee.co.th/3LPmOrdT84</t>
         </is>
       </c>
       <c r="K33" s="2" t="n"/>
       <c r="L33" s="2" t="inlineStr"/>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>WTHB เก้าอี้แคมป์ปิ้ง เพิ่มผ้าฝ้าย พนักพิงสูง เก้าอี้สนาม เก้าอี้สนามพับได้ ปิคนิค รับน้ำหนัก 300KG</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/4fv9z7LZZT</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="n"/>
-      <c r="L34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>ซื้อ 1 แถม1ไฟฉายคาดหัว ไฟคาดหัว ส่องไกล ไฟคาดหัว LED ส่องกบ เดินป่า ลุยฝนได้ สว่างมาก รับประกันความสว่า</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr"/>
-      <c r="D35" s="2" t="inlineStr"/>
-      <c r="E35" s="2" t="inlineStr"/>
-      <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr"/>
-      <c r="H35" s="2" t="inlineStr"/>
-      <c r="I35" s="2" t="inlineStr"/>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/1Vy8DJSgdv</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="n"/>
-      <c r="L35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>20warehouse ไฟฉายคาดศีรษะ LED 90 Lumens ปรับมุมได้ ไฟส่องสว่างพกพา สำหรับเดินป่า กรีดยาง ซ่อมรถ ตกปลา</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/40fTBvEz6Q</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="n"/>
-      <c r="L36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>ซื้อ1แถม1ไฟฉายแรงสูง ไฟฉายLED ไฟฉายพกพา ชาร์จUSB ส่องสว่างไกล ปรับได้5ระดับ</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr"/>
-      <c r="D37" s="2" t="inlineStr"/>
-      <c r="E37" s="2" t="inlineStr"/>
-      <c r="F37" s="2" t="inlineStr"/>
-      <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="inlineStr"/>
-      <c r="I37" s="2" t="inlineStr"/>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/9fJpwLobn1</t>
-        </is>
-      </c>
-      <c r="K37" s="2" t="n"/>
-      <c r="L37" s="2" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>530 Portable Flashlights Miniไฟฉายสว่างมาก CREE LED XPE+COB 2in1 600mah usb charge 3mode ซูมได้</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr"/>
-      <c r="G38" s="2" t="inlineStr"/>
-      <c r="H38" s="2" t="inlineStr"/>
-      <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/2qTVno4nfp</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="n"/>
-      <c r="L38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>เชือกรอกปรับระดับได้ เชือกเต็นท์ เชือกรอกปรับระดับได้ 4m สําหรับตั้งแคมป์กลางแจ้ง รอกเชือก เชือกยก</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr"/>
-      <c r="D39" s="2" t="inlineStr"/>
-      <c r="E39" s="2" t="inlineStr"/>
-      <c r="F39" s="2" t="inlineStr"/>
-      <c r="G39" s="2" t="inlineStr"/>
-      <c r="H39" s="2" t="inlineStr"/>
-      <c r="I39" s="2" t="inlineStr"/>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/1qaybz40f6</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="n"/>
-      <c r="L39" s="2" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>สมอบกเหล็กหล่อ สมอบกเต็นท์ วงแหวนเรืองแสง 20/30/40 CM เหล็กคาร์บอนสูง</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr"/>
-      <c r="G40" s="2" t="inlineStr"/>
-      <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="2" t="inlineStr"/>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/5fnhB2pljE</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="n"/>
-      <c r="L40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>มีดตั้งแคมป์กลางแจ้ง (สแตนเลส) - มีดอเนกประสงค์แบบพกพา คมชัดเป็นพิเศษ G3204</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr"/>
-      <c r="D41" s="2" t="inlineStr"/>
-      <c r="E41" s="2" t="inlineStr"/>
-      <c r="F41" s="2" t="inlineStr"/>
-      <c r="G41" s="2" t="inlineStr"/>
-      <c r="H41" s="2" t="inlineStr"/>
-      <c r="I41" s="2" t="inlineStr"/>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/50Y0Npil9c</t>
-        </is>
-      </c>
-      <c r="K41" s="2" t="n"/>
-      <c r="L41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>#019 Kershaw #Folding knife #มีดพับ #มีดเดินป่า #มีดเอนกประสงค์ LIFEPLAZA</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="2" t="inlineStr"/>
-      <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr"/>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/2gA5bYimaj</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="n"/>
-      <c r="L42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>NANMEEBOOKS หนังสือ แผนที่ประวัติศาสตร์ เหตุการณ์เปลี่ยนโลก เสริมความรู้</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr"/>
-      <c r="D43" s="2" t="inlineStr"/>
-      <c r="E43" s="2" t="inlineStr"/>
-      <c r="F43" s="2" t="inlineStr"/>
-      <c r="G43" s="2" t="inlineStr"/>
-      <c r="H43" s="2" t="inlineStr"/>
-      <c r="I43" s="2" t="inlineStr"/>
-      <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/6Ajxm0MsFI</t>
-        </is>
-      </c>
-      <c r="K43" s="2" t="n"/>
-      <c r="L43" s="2" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>WAYFARER โต๊ะแคมป์กลางแจ้ง โต๊ะพับ โต๊ะไข่เจียว โต๊ะตั้งแคมป์ ซื้อ 1 แถม 1 ถุงจัดส่ง ง่ายต่อการพกพา ทำความสะอาดง่าย</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr"/>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="2" t="inlineStr"/>
-      <c r="H44" s="2" t="inlineStr"/>
-      <c r="I44" s="2" t="inlineStr"/>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/5fnhB6BArU</t>
-        </is>
-      </c>
-      <c r="K44" s="2" t="n"/>
-      <c r="L44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>MAX FIRE แก๊สกระป๋อง แก๊สปิคนิค พร้อมด้วยระบบป้องกันการระเบิด ปริมาณ 250g. ประเทศเกาหลี 1 แพ็ค</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr"/>
-      <c r="D45" s="2" t="inlineStr"/>
-      <c r="E45" s="2" t="inlineStr"/>
-      <c r="F45" s="2" t="inlineStr"/>
-      <c r="G45" s="2" t="inlineStr"/>
-      <c r="H45" s="2" t="inlineStr"/>
-      <c r="I45" s="2" t="inlineStr"/>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/6Ajxm1pku2</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="n"/>
-      <c r="L45" s="2" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>เชือกพาราคอร์ด เชือกตากผ้า เชือก ยาว4/10เมตร เก็บง่าย คุณภาพดี ทนทาน คละสี สำหรับเดินป่า ตั้งแคมป์ ใช้ผูกเอนกประสงค์</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr"/>
-      <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" s="2" t="inlineStr"/>
-      <c r="H46" s="2" t="inlineStr"/>
-      <c r="I46" s="2" t="inlineStr"/>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/AKZWjhSCbh</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="n"/>
-      <c r="L46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>หมอนเป่าลม หมอนหนุนเป่าลมพกพา เบามาก จัดเก็บง่าย ขนาดพกพา 43x28x12cm หมอนเป่าลม ใบใหญ่ เหมาะสำหรับสำนักงาน การท่องเที่ยว</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr"/>
-      <c r="D47" s="2" t="inlineStr"/>
-      <c r="E47" s="2" t="inlineStr"/>
-      <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr"/>
-      <c r="H47" s="2" t="inlineStr"/>
-      <c r="I47" s="2" t="inlineStr"/>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/4qEaBblIDQ</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="n"/>
-      <c r="L47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>ผ้าบัฟ ผ้าโพกหน้า ทั้งวิ่ง ล่าสัตว์ ตกปลา เดินป่า รถจักรยานยนต์ ปั่นจักรยาน เล่นสกี ชิคสุดๆค่าได้ยาวนานคุ้มค่า</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" s="2" t="inlineStr"/>
-      <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="2" t="inlineStr"/>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/3LPmOrdT84</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="n"/>
-      <c r="L48" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L48"/>
+  <autoFilter ref="A1:L33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Rocket21 affiliate pool (2026-08-05 21:52)
</commit_message>
<xml_diff>
--- a/affiliate_data/rocket_curated.xlsx
+++ b/affiliate_data/rocket_curated.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Curated Products" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Curated Products'!$A$1:$L$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Curated Products'!$A$1:$L$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -899,7 +899,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>เก้าอี้แคมป์ปิ้ง พนักพิงสูง เก้าอี้สนาม พับได้ แบบพกพา ปิคนิค แถมถุงเก็บ รับน้ำหนัก 300KG</t>
+          <t>Mobi GARDEN Camping Tarp Flysheet Shelter Sun Shade Anti-UV Canopy กันน้ําปิกนิกกลางแจ้งราคาพิเศษ!</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
@@ -911,7 +911,7 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/AAG6XCsmzJ</t>
+          <t>https://s.shopee.co.th/8AV3flbllA</t>
         </is>
       </c>
       <c r="K18" s="2" t="n"/>
@@ -923,7 +923,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>WTHB เก้าอี้แคมป์ปิ้ง เพิ่มผ้าฝ้าย พนักพิงสูง เก้าอี้สนาม เก้าอี้สนามพับได้ ปิคนิค รับน้ำหนัก 300KG</t>
+          <t>Acebeam TAC 2AA SFT 25R Hi ไฟฉาย LED 1600 ลูเมน 181 เมตรไฟฉาย EDC แบบพกพา USB-C แบตเตอรี่ชาร์จปุ่มคู่ flashligt</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr"/>
@@ -935,7 +935,7 @@
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4fv9z7LZZT</t>
+          <t>https://s.shopee.co.th/4fvBR9C2Q3</t>
         </is>
       </c>
       <c r="K19" s="2" t="n"/>
@@ -947,7 +947,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>ซื้อ 1 แถม1ไฟฉายคาดหัว ไฟคาดหัว ส่องไกล ไฟคาดหัว LED ส่องกบ เดินป่า ลุยฝนได้ สว่างมาก รับประกันความสว่า</t>
+          <t>Swiss TECH-16 in 1 Camping Multitool EDC Multi-Folding Plier Wire Stripper กระเป๋ากลางแจ้งมินิแบบพกพาสําหรับ Camping มาใหม่ล่าสุด</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
@@ -959,7 +959,7 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1Vy8DJSgdv</t>
+          <t>https://s.shopee.co.th/3g2eFG36K8</t>
         </is>
       </c>
       <c r="K20" s="2" t="n"/>
@@ -971,7 +971,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>20warehouse ไฟฉายคาดศีรษะ LED 90 Lumens ปรับมุมได้ ไฟส่องสว่างพกพา สำหรับเดินป่า กรีดยาง ซ่อมรถ ตกปลา</t>
+          <t>Wurkkos TD11 3000lm สมาร์ท OLED ไฟฉายยุทธวิธี, LED RGB ไฟด้านข้างที่มีสีสัน 320-เมตร, สวิตช์คู่, 3.7V 1670mAh แบตเตอรี่ลิเธียม EDC ไฟฉาย</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr"/>
@@ -983,7 +983,7 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/40fTBvEz6Q</t>
+          <t>https://s.shopee.co.th/5fnid02X7w</t>
         </is>
       </c>
       <c r="K21" s="2" t="n"/>
@@ -995,7 +995,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>ซื้อ1แถม1ไฟฉายแรงสูง ไฟฉายLED ไฟฉายพกพา ชาร์จUSB ส่องสว่างไกล ปรับได้5ระดับ</t>
+          <t>SWISS TECH/16 in 1 Camping Multitool, คีมอเนกประสงค์, EDC Wire Stripper, กระเป๋ากลางแจ้ง, มินิแบบพกพาสําหรับ Camping, มาใหม่ล่าสุด</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
@@ -1007,7 +1007,7 @@
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/9fJpwLobn1</t>
+          <t>https://s.shopee.co.th/9V0RBxUr5L</t>
         </is>
       </c>
       <c r="K22" s="2" t="n"/>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>530 Portable Flashlights Miniไฟฉายสว่างมาก CREE LED XPE+COB 2in1 600mah usb charge 3mode ซูมได้</t>
+          <t>MOSSY OAK คีมอเนกประสงค์ 19-in-1 สแตนเลสสตีลเครื่องมือ EDC พร้อมไขควงแขน Self-locking พร้อม Sheath-Perfect สําหรับการตั้งแคมป์กลางแจ้งพร้อมกระเป๋า</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr"/>
@@ -1031,7 +1031,7 @@
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2qTVno4nfp</t>
+          <t>https://s.shopee.co.th/2Vqgr5KnGD</t>
         </is>
       </c>
       <c r="K23" s="2" t="n"/>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>เชือกรอกปรับระดับได้ เชือกเต็นท์ เชือกรอกปรับระดับได้ 4m สําหรับตั้งแคมป์กลางแจ้ง รอกเชือก เชือกยก</t>
+          <t>Sofirn SK1 ไฟฉายยุทธวิธี, 1300 Lumens, กันน้ํา IP68, โยนยาว, ชาร์จใหม่ได้, EDC</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
@@ -1055,7 +1055,7 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/1qaybz40f6</t>
+          <t>https://s.shopee.co.th/40fUdy84Q9</t>
         </is>
       </c>
       <c r="K24" s="2" t="n"/>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>สมอบกเหล็กหล่อ สมอบกเต็นท์ วงแหวนเรืองแสง 20/30/40 CM เหล็กคาร์บอนสูง</t>
+          <t>NEXTORCH NP12 Ti EDC ปากกาลูกปัดเซรามิคแก้ว Breaker หัวไทเทเนียมปากกาการอยู่รอดฉุกเฉิน Self-defense</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr"/>
@@ -1079,7 +1079,7 @@
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5fnhB2pljE</t>
+          <t>https://s.shopee.co.th/7fYn0i2Qis</t>
         </is>
       </c>
       <c r="K25" s="2" t="n"/>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>มีดตั้งแคมป์กลางแจ้ง (สแตนเลส) - มีดอเนกประสงค์แบบพกพา คมชัดเป็นพิเศษ G3204</t>
+          <t>จัดส่งจากกรุงเทพVOTAGOO กระเป๋าเอวทัคติคอล EDC พกพา ผ้าไนลอน420D ทนทาน ซิปYKK แขนงค์Duraflex กระเป๋าใส่อุปกรณ์กลางแจ้ง ความจุ7ลิตร PISTOL WAIST PACKCOD)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr"/>
@@ -1103,7 +1103,7 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/50Y0Npil9c</t>
+          <t>https://s.shopee.co.th/50Y1poTySo</t>
         </is>
       </c>
       <c r="K26" s="2" t="n"/>
@@ -1115,7 +1115,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>#019 Kershaw #Folding knife #มีดพับ #มีดเดินป่า #มีดเอนกประสงค์ LIFEPLAZA</t>
+          <t>กระเป๋าสะพายข้าง edc compact shoulder helikon codura</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr"/>
@@ -1127,7 +1127,7 @@
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/2gA5bYimaj</t>
+          <t>https://s.shopee.co.th/50Y1psApQp</t>
         </is>
       </c>
       <c r="K27" s="2" t="n"/>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>NANMEEBOOKS หนังสือ แผนที่ประวัติศาสตร์ เหตุการณ์เปลี่ยนโลก เสริมความรู้</t>
+          <t>Naturehike lw180 ถุงนอนผ้าฝ้าย น้ําหนักเบา สําหรับตั้งแคมป์ เดินป่า กลางแจ้ง แผ่นรองนอน</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr"/>
@@ -1151,7 +1151,7 @@
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6Ajxm0MsFI</t>
+          <t>https://s.shopee.co.th/2qTXGB3YXk</t>
         </is>
       </c>
       <c r="K28" s="2" t="n"/>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>WAYFARER โต๊ะแคมป์กลางแจ้ง โต๊ะพับ โต๊ะไข่เจียว โต๊ะตั้งแคมป์ ซื้อ 1 แถม 1 ถุงจัดส่ง ง่ายต่อการพกพา ทำความสะอาดง่าย</t>
+          <t>เข็มขัด Rattler EDC Belt เข็มขัดแบบใส่ได้ทุกวันสไตล์แทคติคอล</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr"/>
@@ -1175,7 +1175,7 @@
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/5fnhB6BArU</t>
+          <t>https://s.shopee.co.th/AKZYBgqbOA</t>
         </is>
       </c>
       <c r="K29" s="2" t="n"/>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>MAX FIRE แก๊สกระป๋อง แก๊สปิคนิค พร้อมด้วยระบบป้องกันการระเบิด ปริมาณ 250g. ประเทศเกาหลี 1 แพ็ค</t>
+          <t>เข็มขัดไนลอน EDC ทรงแข็ง GUNBANGKOK | หัวล็อคออโต้ แข็งแรง ปรับได้ Free Size</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr"/>
@@ -1199,7 +1199,7 @@
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/6Ajxm1pku2</t>
+          <t>https://s.shopee.co.th/2Vqgr7kJbX</t>
         </is>
       </c>
       <c r="K30" s="2" t="n"/>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>เชือกพาราคอร์ด เชือกตากผ้า เชือก ยาว4/10เมตร เก็บง่าย คุณภาพดี ทนทาน คละสี สำหรับเดินป่า ตั้งแคมป์ ใช้ผูกเอนกประสงค์</t>
+          <t>MODOFO ที่นอนลม มีหมอน ที่นอนลมกลางแจ้ง เบาะนอนพกพา 190*60ซม เตียงเป่าลม ที่แคมป์ปิ้ง พกพาสะดวก</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr"/>
@@ -1223,7 +1223,7 @@
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/AKZWjhSCbh</t>
+          <t>https://s.shopee.co.th/7AcWQ5s3Jr</t>
         </is>
       </c>
       <c r="K31" s="2" t="n"/>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>หมอนเป่าลม หมอนหนุนเป่าลมพกพา เบามาก จัดเก็บง่าย ขนาดพกพา 43x28x12cm หมอนเป่าลม ใบใหญ่ เหมาะสำหรับสำนักงาน การท่องเที่ยว</t>
+          <t>WOLF EDC รอกตกปลา เฟืองทองเหลือง 6BB ระบบ Digital Control คลิ๊กเสียงปลาลาก ตกปลา รอกหยดน้ำ รอกเบท</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr"/>
@@ -1247,7 +1247,7 @@
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/4qEaBblIDQ</t>
+          <t>https://s.shopee.co.th/9fJrOK5EOc</t>
         </is>
       </c>
       <c r="K32" s="2" t="n"/>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>ผ้าบัฟ ผ้าโพกหน้า ทั้งวิ่ง ล่าสัตว์ ตกปลา เดินป่า รถจักรยานยนต์ ปั่นจักรยาน เล่นสกี ชิคสุดๆค่าได้ยาวนานคุ้มค่า</t>
+          <t>หนาขึ้น20เท่าPIKA ผ้าเต้นท์ หนา6800D (เฉพาะผ้า)ผ้าใบเต็นท์ กันน้ำ กันแดด กันยูวี 2x2 2x3 3x3 เต็นท์พับได้ เต็นท์ขายของ</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr"/>
@@ -1271,14 +1271,470 @@
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>https://s.shopee.co.th/3LPmOrdT84</t>
+          <t>https://s.shopee.co.th/5fn14DklSQ</t>
         </is>
       </c>
       <c r="K33" s="2" t="n"/>
       <c r="L33" s="2" t="inlineStr"/>
     </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Wurkkos ไฟ EDC WK03 1800lm SST40 USB C ชาร์จซ้ําได้ 18650 UI พร้อมตัวบ่งชี้พลังงาน ATR</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4qEbdNtq5O</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="n"/>
+      <c r="L34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>เก้าอี้แคมป์ปิ้ง คนอ้วน พร้อมกระเป๋าจัดเก็บ โครงอลูมิเนียมรับน้ำหนักได้ 300KG</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9V0RCM6764</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="n"/>
+      <c r="L35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>เปลญวน เก้าอี้ชิงช้า แบบแขวน เก้าอี้นั่งทรงกลม แบบถักแฮนด์เมด สไตล์นอร์ดิก</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7psDDO1ANv</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="n"/>
+      <c r="L36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>PIKA ผ้าเต้นท์ หนาสุดๆ6800D(เฉพาะผ้า)กันน้ำ กันยูวี100% ผ้าใบเต็นท์ เต็นท์ขายของ 2x2 2x3 3x3เมตร ผ้าสวยถูกใจแน่นอน</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/3VjE3KKyrA</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="n"/>
+      <c r="L37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>มัลติทูลอเนกประสงค์ TRAVELER ของแท้ 12in1 สีขาว แบบพกพา มีระบบล๊อก EDC แคมป์ปิ้ง ติดรถ งานช่าง มีเลื่อย ไขควง</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/30mxS448y2</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="n"/>
+      <c r="L38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Leacat กระเป๋าเป้สะพายหลัง EDC กันน้ํา ขนาด 20 ลิตร สําหรับเดินป่า ล่าสัตว์</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr"/>
+      <c r="D39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7AcWPiY7uJ</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="n"/>
+      <c r="L39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Free hike เก้าอี้แคมป์ปิ้ง เก้าอี้สนามที่พับได้ camping ขาตั้งอลูมิเนียม รับน้ำหนักได้ 300กก</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9Kh103XYhh</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="n"/>
+      <c r="L40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>COD เตาแอลกอฮอล์ เตาแอลกอฮอล์สแตนเลสแบบพกพา เตาตั้งแคมป์สําหรับตั้งแคมป์</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr"/>
+      <c r="D41" s="2" t="inlineStr"/>
+      <c r="E41" s="2" t="inlineStr"/>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/gP2g8D94P</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="n"/>
+      <c r="L41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>ห่วงตัวดี ไทเทเนียม ห่วงเกือกม้า Titanium D-Shackle พร้อมสกรูถอดประกอบ สำหรับพวงกุญแจ EDC มี 2 ขนาด 12mm 17mm</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/3B6NePzLDc</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="n"/>
+      <c r="L42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>PKT ยางนอกไม่ใช้ยางใน(Tubeless) ขอบ12,13,14,15,10 ZOOMER X,PCX,GRAND FILANO,NMAX พีเคที ยางไทยแท้</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr"/>
+      <c r="D43" s="2" t="inlineStr"/>
+      <c r="E43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/2VqgqGBUTJ</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="n"/>
+      <c r="L43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>MDช่องหลัก นีออนหัวเชื้อสลายคราบช่วงล่าง คราบน้ำมันคราบฝังแน่น คราบฝังตามล้อยาง</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8V7tzwBGOA</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="n"/>
+      <c r="L44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>ผ้าคลุมรถมอเตอร์ไซค์ กันน้ำ กันฝุ่น กันแดด หนา 5 ชั้น วัสดุทนทาน สีดำ ขนาด M/ L / XL / XXL</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr"/>
+      <c r="D45" s="2" t="inlineStr"/>
+      <c r="E45" s="2" t="inlineStr"/>
+      <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/111t3VPrXd</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="n"/>
+      <c r="L45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>หมวกกันน๊อค motorcycle helmet ส่งจากกทม. COD ได้ เลนส์คู่ กันแดด ระบายอากาศ ABS แข็งแรง</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7VFMnV46DI</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="n"/>
+      <c r="L46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>FOAMING CLEANER ผลิตภัณฑ์ทำความสะอาดในรถยนต์ เบาะ คอนโซล พรมปูพื้นรถยนต์</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr"/>
+      <c r="D47" s="2" t="inlineStr"/>
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/2LXGeccjdi</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="n"/>
+      <c r="L47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>KATHWI น้ําหอมติดรถยนต์ K-nature, Rose Forest, Yu Long Tea, Eternal Water Balm, กลิ่นหอมติดทนนานและน่ารื่นรมย์, น้ําหอมติดรถยนต์สุดหรูล่าสุด 180g</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9Kh0zPnAOe</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="n"/>
+      <c r="L48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>ENDURO 4T RACING 10W-40 ขนาด 0.8L น้ำมันเครื่องรถจักรยานยนต์ 4 จังหวะคุณภาพสูง</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr"/>
+      <c r="D49" s="2" t="inlineStr"/>
+      <c r="E49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4VblDqEpBe</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="n"/>
+      <c r="L49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Nano Ceramic Window Film ฟิล์มกรองแสงรถยนต์ ฟิล์มกรองแสง ฟิล์มอาคาร เซรามิค (ราคาต่อเมตร)</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr"/>
+      <c r="H50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/3B6Ne6CETd</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="n"/>
+      <c r="L50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>TwoStar เสื้อแจ็คเก็ตบอมเบอร์เรียบๆ สำหรับผู้ชายและผู้หญิง คุณภาพสูง เสื้อโค้ททรงมอเตอร์ไซค์ คอกลม ขนาดกำลังดี</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr"/>
+      <c r="D51" s="2" t="inlineStr"/>
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="inlineStr"/>
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/20uQFIeFPs</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="n"/>
+      <c r="L51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>หัวฉีดเเต่ง 6รู J 125CC 150CC(สั้น) 6รู G 145 150CC 8รูJ W 170CC(สั้น) ใส่กับ click125i wave110i new KZR คลิก125ไอ KYZ</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/3LPnplDFaz</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="n"/>
+      <c r="L52" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L33"/>
+  <autoFilter ref="A1:L52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>